<commit_message>
Update BNY contacts after profile verification
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1112,19 +1112,21 @@
       </c>
       <c r="S8" s="43" t="inlineStr">
         <is>
-          <t>Sonia Kataria — Engineering Strategy and Execution, Office of the CIO and CFO
-Nathan Whittall — Lead Analyst, FinOps (уже в команде)</t>
+          <t>Eli Grinvald — Head of Cloud, BNY Mellon | PershingX (владелец облака; проверено по профилю)
+Katie Sealander Skavronski — SVP, FP&amp;A, Technology Finance (финансы технологий; проверено по профилю)
+Sonia Kataria — COO, Technology, Strategy &amp; Execution, Office of the CIO (союзник на уровне CIO/CFO; проверено по профилю)</t>
         </is>
       </c>
       <c r="T8" s="43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/sonia-kataria-ny
-https://www.linkedin.com/in/nathan-whittall-538081145</t>
+          <t>https://www.linkedin.com/in/eligrinvald
+https://www.linkedin.com/in/katie-sealander-skavronski
+https://www.linkedin.com/in/sonia-kataria-ny</t>
         </is>
       </c>
       <c r="U8" s="43" t="inlineStr">
         <is>
-          <t>Соня — ближайшее совпадение с «CFO, Engineering»; проверить, что она и есть руководитель. Nathan — рядовой аналитик, использовать как вход, не как ЛПР. Hub Lead в Seamless не найден.</t>
+          <t>Порядок: Eli, затем Katie, затем Sonia, не в один день. Никто из троих не подтверждён как руководитель вакансии. Nathan Whittall убран: его «FinOps» — клиентский биллинг BNY Pershing. Engineering Hub Lead в Seamless не найден. Для Eli в письме можно упомянуть Kubernetes (cluster-level, поды, контейнеры, рекомендации) — подтверждено коллегой, проверить объём пилота.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update HealthEdge contacts after profile verification
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1210,19 +1210,20 @@
       </c>
       <c r="S9" s="43" t="inlineStr">
         <is>
-          <t>James Fallon — VP, Cloud Infrastructure &amp; Operations
-Philip Anzalone — SVP Finance</t>
+          <t>James Fallon — VP, Cloud Infrastructure &amp; Operations, HealthEdge (владелец облака, портфель $40M+, запускал FinOps-программы, отчитывается CEO/CFO/CTO; проверено по профилю)
+Дополнительно, не проверено: Philip Anzalone — SVP Finance; Matt Mclaughlin — CFO</t>
         </is>
       </c>
       <c r="T9" s="43" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/james-fallon-cissp-ccsk
-https://www.linkedin.com/in/philip-anzalone-1b508a18</t>
+https://www.linkedin.com/in/philip-anzalone-1b508a18
+https://www.linkedin.com/in/matt-mclaughlin-36b7bb4</t>
         </is>
       </c>
       <c r="U9" s="43" t="inlineStr">
         <is>
-          <t>Подчинение в вакансии не указано. FinOps-специалистов в базе нет. Первый — владелец облака, второй — финансы. Также CFO: Matt Mclaughlin https://www.linkedin.com/in/matt-mclaughlin-36b7bb4</t>
+          <t>Вероятный руководитель вакансии (подчинение в вакансии не указано). Бюджет подтверждён профилем ($40M+ мультиоблако). Опытный в FinOps: письмо короткое, с вопросом. Конкурентный инструмент в профиле не назван. Про расходы по клиентам/функциям продукта не обещать, пока не подтверждено.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify Philip Anzalone and set HealthEdge outreach order
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1210,8 +1210,9 @@
       </c>
       <c r="S9" s="43" t="inlineStr">
         <is>
-          <t>James Fallon — VP, Cloud Infrastructure &amp; Operations, HealthEdge (владелец облака, портфель $40M+, запускал FinOps-программы, отчитывается CEO/CFO/CTO; проверено по профилю)
-Дополнительно, не проверено: Philip Anzalone — SVP Finance; Matt Mclaughlin — CFO</t>
+          <t>1) James Fallon — VP, Cloud Infrastructure &amp; Operations (владелец облака, портфель $40M+, запускал FinOps-программы; проверено по профилю)
+2) Philip Anzalone — SVP Finance (бюджеты $100M+, моделирование рентабельности продуктов; проверено по профилю)
+Не проверено: Matt Mclaughlin — CFO</t>
         </is>
       </c>
       <c r="T9" s="43" t="inlineStr">
@@ -1223,7 +1224,7 @@
       </c>
       <c r="U9" s="43" t="inlineStr">
         <is>
-          <t>Вероятный руководитель вакансии (подчинение в вакансии не указано). Бюджет подтверждён профилем ($40M+ мультиоблако). Опытный в FinOps: письмо короткое, с вопросом. Конкурентный инструмент в профиле не назван. Про расходы по клиентам/функциям продукта не обещать, пока не подтверждено.</t>
+          <t>Порядок: James, через 3–5 дней Philip, CFO — только после ответа. James — вероятный руководитель вакансии (подчинение в вакансии не указано), Philip — финансовый партнёр. Расходы по продукту/команде/владельцу можно обещать (подтверждено); по клиентам и функциям продукта — нет.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark HealthEdge CFO as escalation contact
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1212,7 +1212,7 @@
         <is>
           <t>1) James Fallon — VP, Cloud Infrastructure &amp; Operations (владелец облака, портфель $40M+, запускал FinOps-программы; проверено по профилю)
 2) Philip Anzalone — SVP Finance (бюджеты $100M+, моделирование рентабельности продуктов; проверено по профилю)
-Не проверено: Matt Mclaughlin — CFO</t>
+3) Matt McLaughlin — CFO с 2021 (проверено по профилю; эскалация, не первый контакт)</t>
         </is>
       </c>
       <c r="T9" s="43" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="U9" s="43" t="inlineStr">
         <is>
-          <t>Порядок: James, через 3–5 дней Philip, CFO — только после ответа. James — вероятный руководитель вакансии (подчинение в вакансии не указано), Philip — финансовый партнёр. Расходы по продукту/команде/владельцу можно обещать (подтверждено); по клиентам и функциям продукта — нет.</t>
+          <t>Порядок: James, через 3–5 дней Philip, CFO Matt McLaughlin — только после ответа James/Philip или если оба молчат после двух попыток (повестка в его постах: маржа и рост затрат). James — вероятный руководитель вакансии (подчинение в вакансии не указано), Philip — финансовый партнёр. Расходы по продукту/команде/владельцу можно обещать (подтверждено); по клиентам и функциям продукта — нет.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify Charlie Piazza for Ochsner
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1308,19 +1308,21 @@
       </c>
       <c r="S10" s="43" t="inlineStr">
         <is>
-          <t>Charlie Piazza — Director, Public Cloud &amp; Data Services
-Jack McLeod — AVP, Hybrid Cloud Services</t>
+          <t>1) Charlie Piazza — Director, Public Cloud &amp; Data Services (владелец облака, в Ochsner с 2017; проверено по профилю; не руководитель вакансии)
+Не проверено: Jack McLeod — AVP, Hybrid Cloud Services; Amy Trainor — SVP &amp; CIO
+НЕ НАЙДЕН: Technology Business Manager (руководитель вакансии) — искать вручную в LinkedIn</t>
         </is>
       </c>
       <c r="T10" s="43" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/charlie-piazza-86b03127
-https://www.linkedin.com/in/jackmcleod</t>
+https://www.linkedin.com/in/jackmcleod
+https://www.linkedin.com/in/amy-trainor-rn-7858b61b</t>
         </is>
       </c>
       <c r="U10" s="43" t="inlineStr">
         <is>
-          <t>Technology Business Manager в Seamless не найден — искать вручную в LinkedIn. CIO: Amy Trainor https://www.linkedin.com/in/amy-trainor-rn-7858b61b</t>
+          <t>Если TBM найдётся — писать ему первым, Charlie вторым. В письме Charlie просим указать, кто отвечает за подотчётность затрат. Snowflake не упоминать (возможности не подтверждены).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Eric DiZinno as lead Ochsner contact
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1308,21 +1308,23 @@
       </c>
       <c r="S10" s="43" t="inlineStr">
         <is>
-          <t>1) Charlie Piazza — Director, Public Cloud &amp; Data Services (владелец облака, в Ochsner с 2017; проверено по профилю; не руководитель вакансии)
+          <t>1) Eric DiZinno — VP Finance, IS and Connected Health (финансовый владелец IT/digital; с 02.2026, 16 лет в Ochsner; проверено по профилю)
+2) Charlie Piazza — Director, Public Cloud &amp; Data Services (владелец облака; проверено по профилю)
 Не проверено: Jack McLeod — AVP, Hybrid Cloud Services; Amy Trainor — SVP &amp; CIO
-НЕ НАЙДЕН: Technology Business Manager (руководитель вакансии) — искать вручную в LinkedIn</t>
+НЕ НАЙДЕН: Technology Business Manager (руководитель вакансии) — в LinkedIn-поиске по Ochsner нет; смотреть Meet the hiring team в вакансии</t>
         </is>
       </c>
       <c r="T10" s="43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/charlie-piazza-86b03127
+          <t>https://www.linkedin.com/in/eric-dizinno-983408147
+https://www.linkedin.com/in/charlie-piazza-86b03127
 https://www.linkedin.com/in/jackmcleod
 https://www.linkedin.com/in/amy-trainor-rn-7858b61b</t>
         </is>
       </c>
       <c r="U10" s="43" t="inlineStr">
         <is>
-          <t>Если TBM найдётся — писать ему первым, Charlie вторым. В письме Charlie просим указать, кто отвечает за подотчётность затрат. Snowflake не упоминать (возможности не подтверждены).</t>
+          <t>Порядок: Eric, через 3–5 дней Charlie. В письме Eric просим указать, кто отвечает за облачные расходы (выход на TBM); в письме Charlie эту просьбу заменить. Snowflake не упоминать (возможности не подтверждены).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Jack McLeod to Ochsner contacts and set order
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1308,23 +1308,24 @@
       </c>
       <c r="S10" s="43" t="inlineStr">
         <is>
-          <t>1) Eric DiZinno — VP Finance, IS and Connected Health (финансовый владелец IT/digital; с 02.2026, 16 лет в Ochsner; проверено по профилю)
-2) Charlie Piazza — Director, Public Cloud &amp; Data Services (владелец облака; проверено по профилю)
-Не проверено: Jack McLeod — AVP, Hybrid Cloud Services; Amy Trainor — SVP &amp; CIO
+          <t>1) Eric DiZinno — VP Finance, IS and Connected Health (финансовый владелец IT/digital; проверено по профилю)
+2) Jack McLeod — AVP, Hybrid Cloud Services (стратегия гибридного облака, с 07.2025, ex-Accenture/Trace3; проверено по профилю)
+3) Charlie Piazza — Director, Public Cloud &amp; Data Services (владелец облака; возможно, подчиняется Jack; проверено по профилю)
+Не проверено: Amy Trainor — SVP &amp; CIO
 НЕ НАЙДЕН: Technology Business Manager (руководитель вакансии) — в LinkedIn-поиске по Ochsner нет; смотреть Meet the hiring team в вакансии</t>
         </is>
       </c>
       <c r="T10" s="43" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/eric-dizinno-983408147
+https://www.linkedin.com/in/jackmcleod
 https://www.linkedin.com/in/charlie-piazza-86b03127
-https://www.linkedin.com/in/jackmcleod
 https://www.linkedin.com/in/amy-trainor-rn-7858b61b</t>
         </is>
       </c>
       <c r="U10" s="43" t="inlineStr">
         <is>
-          <t>Порядок: Eric, через 3–5 дней Charlie. В письме Eric просим указать, кто отвечает за облачные расходы (выход на TBM); в письме Charlie эту просьбу заменить. Snowflake не упоминать (возможности не подтверждены).</t>
+          <t>Порядок: Eric, через 3–5 дней Jack, ещё через 3–5 дней Charlie. Просьбу «указать, кто отвечает» оставить только в письме Eric. Snowflake не упоминать. В письме Jack пилот ограничен AWS/Azure: покрытие частных платформ/дата-центров не подтверждено; Kubernetes упомянут условно.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Stride row: no suitable contact found yet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1409,17 +1409,18 @@
       </c>
       <c r="S11" s="43" t="inlineStr">
         <is>
-          <t>Praveen Vegesna — Senior DevOps / FinOps (возможно, уже действующий FinOps-специалист)</t>
+          <t>НЕТ ПОДХОДЯЩЕГО КОНТАКТА. Praveen Vegesna — Sr. DevOps/FinOps, подрядчик (Contract) с 04.2025, значок Open to work (проверено по профилю): не покупатель, писать не стоит.
+Руководители облака/инфраструктуры в Seamless не найдены (поиск по stridelearning.com дал маркетинг, корп. развитие и инженеров).</t>
         </is>
       </c>
       <c r="T11" s="43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/praveen-vegesna-24b6744a</t>
+          <t>(искать вручную; для справки) https://www.linkedin.com/in/praveen-vegesna-24b6744a</t>
         </is>
       </c>
       <c r="U11" s="43" t="inlineStr">
         <is>
-          <t>Руководители облака/инфраструктуры в Seamless не найдены (поиск по stridelearning.com пуст). Остальные результаты — security-инженеры.</t>
+          <t>Низкий приоритет, вернуться после других компаний. Искать вручную в LinkedIn: Meet the hiring team в вакансии; CIO/CTO/VP Infrastructure/VP Cloud/Director IT Finance в Stride, Inc. Open to work у подрядчика может означать конец контракта и найм штатного FinOps (вакансия актуальна).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Stride contacts after profile checks
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1409,18 +1409,20 @@
       </c>
       <c r="S11" s="43" t="inlineStr">
         <is>
-          <t>НЕТ ПОДХОДЯЩЕГО КОНТАКТА. Praveen Vegesna — Sr. DevOps/FinOps, подрядчик (Contract) с 04.2025, значок Open to work (проверено по профилю): не покупатель, писать не стоит.
-Руководители облака/инфраструктуры в Seamless не найдены (поиск по stridelearning.com дал маркетинг, корп. развитие и инженеров).</t>
+          <t>1) Sinduja Rajagopalan — FP&amp;A Manager, Corporate FP&amp;A (Technology, Product and Strategic Finance); 5 лет в Stride; проверено по профилю. Вход через финансы, не ЛПР.
+Не проверено: Rich Maye — VP Information Technology (работает ли в Stride — неясно); Levon Hooks — CIO (в заголовке fractional/Open to Board); Donna Blackman — CFO (эскалация).
+Отклонены после проверки: Jen H. (Director GRC — безопасность/комплаенс, не расходы); Praveen Vegesna (подрядчик, Open to work).
+Руководитель вакансии не найден.</t>
         </is>
       </c>
       <c r="T11" s="43" t="inlineStr">
         <is>
-          <t>(искать вручную; для справки) https://www.linkedin.com/in/praveen-vegesna-24b6744a</t>
+          <t>Ссылок на профили нет (были только скриншоты): добавить вручную из LinkedIn — Sinduja Rajagopalan (проверена), Levon Hooks, Rich Maye, Donna Blackman (не проверены)</t>
         </is>
       </c>
       <c r="U11" s="43" t="inlineStr">
         <is>
-          <t>Низкий приоритет, вернуться после других компаний. Искать вручную в LinkedIn: Meet the hiring team в вакансии; CIO/CTO/VP Infrastructure/VP Cloud/Director IT Finance в Stride, Inc. Open to work у подрядчика может означать конец контракта и найм штатного FinOps (вакансия актуальна).</t>
+          <t>Порядок: Sinduja (просим назвать, кто владеет облачными затратами) -&gt; Rich Maye/Levon Hooks после проверки профилей -&gt; CFO для эскалации. Низкий приоритет относительно других компаний.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Sinduja link and verify Sandeep P. at Stifel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1417,7 +1417,8 @@
       </c>
       <c r="T11" s="43" t="inlineStr">
         <is>
-          <t>Ссылок на профили нет (были только скриншоты): добавить вручную из LinkedIn — Sinduja Rajagopalan (проверена), Levon Hooks, Rich Maye, Donna Blackman (не проверены)</t>
+          <t>Sinduja Rajagopalan (проверена): https://www.linkedin.com/in/sindujarajagopalan/
+Не проверены, ссылки добавить из LinkedIn: Levon Hooks, Rich Maye, Donna Blackman</t>
         </is>
       </c>
       <c r="U11" s="43" t="inlineStr">
@@ -1506,21 +1507,21 @@
       </c>
       <c r="S12" s="43" t="inlineStr">
         <is>
-          <t>Lauren Borik — FinOps Specialist (с 06.2026)
-Mithun Ayachit — Director, Cloud Strategy and Engineering</t>
+          <t>1) Sandeep P. — Product Management, Stifel Financial (с 06.2024; владеет стратегией и roadmap корпоративной AWS-инфраструктуры, ведёт FinOps по всему облаку, отношения с AWS/AMS, AI-инфраструктура SageMaker/Bedrock; проверено по профилю; это исходная ссылка из таблицы)
+Не проверены: Mithun Ayachit — Director, Cloud Strategy and Engineering; Lauren Borik — FinOps Specialist (с 06.2026); вторая исходная ссылка (shanecredille)</t>
         </is>
       </c>
       <c r="T12" s="44" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/sandeep-p-581ab64/
-https://www.linkedin.com/in/shanecredille/
+https://www.linkedin.com/in/mithunayachit
 https://www.linkedin.com/in/lauren-borik-396702225
-https://www.linkedin.com/in/mithunayachit</t>
+https://www.linkedin.com/in/shanecredille/</t>
         </is>
       </c>
       <c r="U12" s="43" t="inlineStr">
         <is>
-          <t>Две исходные ссылки не менялись и в Seamless не проверялись по имени. Mithun — вероятный руководитель по облаку, проверить.</t>
+          <t>Первый: Sandeep P. (практик FinOps и владелец AWS, вероятно, одна из «старших специалистов FinOps», кому подчиняется роль). Команда FinOps уже есть — это расширение; у Sandeep вероятно есть процессы и, возможно, инструмент: письмо с вопросом про атрибуцию по владельцам. Остальные проверять по профилям.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Flag MetLife contact Rob Fewkes as moved to WTW
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1605,17 +1605,21 @@
       </c>
       <c r="S13" s="43" t="inlineStr">
         <is>
-          <t>Rob Fewkes — Head of Cloud Business Office, Global Technology</t>
+          <t>Rob Fewkes — НЕ ПОДХОДИТ для MetLife: ушёл из MetLife в 02.2026, сейчас Head of Cost Optimization – Global Technology, WTW (проверено по профилю; Seamless устарел).
+Не проверены (могут быть устаревшими): Heather Ratkowiak — Portfolio Manager, Cloud Business Office; Patricia Johnson-Clifton — Principal, Cloud Business Office.
+НУЖЕН: актуальный руководитель Cloud Business Office MetLife — искать вручную в LinkedIn.</t>
         </is>
       </c>
       <c r="T13" s="43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/robfewkes</t>
+          <t>https://www.linkedin.com/in/heatherratkowiak (не проверена)
+https://www.linkedin.com/in/patricia-johnson-clifton-6488675 (не проверена)
+Rob Fewkes (для справки, WTW): https://www.linkedin.com/in/robfewkes</t>
         </is>
       </c>
       <c r="U13" s="43" t="inlineStr">
         <is>
-          <t>Прямое совпадение с «Cloud Business Office». Также в офисе: Heather Ratkowiak (Portfolio Manager) https://www.linkedin.com/in/heatherratkowiak</t>
+          <t>Данные Seamless по MetLife устарели. Освободившаяся роль главы Cloud Business Office может быть связана с вакансией Cloud FinOps Analyst. Rob Fewkes — отдельная возможная цель в WTW, но WTW — консалтинг/брокер (по документу консалтинг исключён): решить отдельно.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify Leroy Straker as lead MetLife contact
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1605,21 +1605,23 @@
       </c>
       <c r="S13" s="43" t="inlineStr">
         <is>
-          <t>Rob Fewkes — НЕ ПОДХОДИТ для MetLife: ушёл из MetLife в 02.2026, сейчас Head of Cost Optimization – Global Technology, WTW (проверено по профилю; Seamless устарел).
-Не проверены (могут быть устаревшими): Heather Ratkowiak — Portfolio Manager, Cloud Business Office; Patricia Johnson-Clifton — Principal, Cloud Business Office.
-НУЖЕН: актуальный руководитель Cloud Business Office MetLife — искать вручную в LinkedIn.</t>
+          <t>1) Leroy Straker — Director, Cloud Business Office, MetLife (с 02.2026, преемник Rob Fewkes; 11,5 лет в MetLife; в About: Cloud FinOps, TBM, FP&amp;A, FinOps Certified Practitioner; проверено по профилю). Руководитель вакансии и владелец функции.
+2) Patricia Johnson-Clifton — Principal, Cloud Business Office (текущая по LinkedIn-выдаче; на фото рамка Open to work — проверить)
+3) Heather R. (Ratkowiak) — Portfolio Manager, Cloud Business Office (текущая; низкий приоритет)
+Rob Fewkes — НЕ подходит для MetLife: ушёл в WTW 02.2026.</t>
         </is>
       </c>
       <c r="T13" s="43" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/heatherratkowiak (не проверена)
-https://www.linkedin.com/in/patricia-johnson-clifton-6488675 (не проверена)
-Rob Fewkes (для справки, WTW): https://www.linkedin.com/in/robfewkes</t>
+          <t>Leroy Straker: ссылку добавить из LinkedIn (были только скриншоты)
+https://www.linkedin.com/in/patricia-johnson-clifton-6488675
+https://www.linkedin.com/in/heatherratkowiak
+(Rob Fewkes, WTW, для справки) https://www.linkedin.com/in/robfewkes</t>
         </is>
       </c>
       <c r="U13" s="43" t="inlineStr">
         <is>
-          <t>Данные Seamless по MetLife устарели. Освободившаяся роль главы Cloud Business Office может быть связана с вакансией Cloud FinOps Analyst. Rob Fewkes — отдельная возможная цель в WTW, но WTW — консалтинг/брокер (по документу консалтинг исключён): решить отдельно.</t>
+          <t>Порядок: Leroy, через 3–5 дней Patricia (проверить Open to work). Вопрос в письме — как сейчас делают привязку затрат к приложению/владельцу. Возможный инструмент TBM/FinOps не назван — узнать на звонке (конкурент = второй эшелон). Rob Fewkes в WTW — решить отдельно (консалтинг/брокер исключён по документу).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Edward Jones to second tier
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -293,7 +293,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -444,6 +444,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -4320,6 +4329,33 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="110" customHeight="1" s="26">
+      <c r="A8" s="53" t="inlineStr">
+        <is>
+          <t>Edward Jones</t>
+        </is>
+      </c>
+      <c r="B8" s="54" t="inlineStr">
+        <is>
+          <t>Senior Digital Product Owner (FinOps)</t>
+        </is>
+      </c>
+      <c r="C8" s="55" t="inlineStr">
+        <is>
+          <t>26.09.2026 (1 нед.)</t>
+        </is>
+      </c>
+      <c r="D8" s="55" t="inlineStr">
+        <is>
+          <t>Fortune 500, 20 000 консультантов, St. Louis; крупные облачные расходы; ищут владельца FinOps-продукта: распределение затрат, showback/chargeback, коммитменты (reservations, savings plans), роль связана со service owners и CSDM. Возможный контакт: Kevin Krueger (Head of Cloud Business Office, не проверен по профилю)</t>
+        </is>
+      </c>
+      <c r="E8" s="55" t="inlineStr">
+        <is>
+          <t>«Mature FinOps organization» (не создают практику); в требованиях опыт с Cloudability/CloudHealth — вероятен конкурент; CSDM = ServiceNow CMDB; облака названы расплывчато (Azure + другие). Оценка по критериям ≈5 из 10</t>
+        </is>
+      </c>
+    </row>
     <row r="9" ht="30" customHeight="1" s="26">
       <c r="A9" s="52" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Verify Kevin Krueger for Edward Jones
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -4329,7 +4329,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="110" customHeight="1" s="26">
+    <row r="8" ht="150" customHeight="1" s="26">
       <c r="A8" s="53" t="inlineStr">
         <is>
           <t>Edward Jones</t>
@@ -4347,12 +4347,13 @@
       </c>
       <c r="D8" s="55" t="inlineStr">
         <is>
-          <t>Fortune 500, 20 000 консультантов, St. Louis; крупные облачные расходы; ищут владельца FinOps-продукта: распределение затрат, showback/chargeback, коммитменты (reservations, savings plans), роль связана со service owners и CSDM. Возможный контакт: Kevin Krueger (Head of Cloud Business Office, не проверен по профилю)</t>
+          <t>Fortune 500, 20 000 консультантов, St. Louis; крупные облачные расходы; роль: распределение затрат, showback/chargeback, коммитменты (reservations, savings plans), service owners и CSDM.
+Контакт: Kevin Krueger — Head of Cloud Business Office (с 08.2024; 10+ лет FinOps/TBM; сам нанимает на «growing and maturing FinOps program»; проверено по профилю). Репостнул вакансию Managing Director, Head of Cloud — возможно, его руководитель.</t>
         </is>
       </c>
       <c r="E8" s="55" t="inlineStr">
         <is>
-          <t>«Mature FinOps organization» (не создают практику); в требованиях опыт с Cloudability/CloudHealth — вероятен конкурент; CSDM = ServiceNow CMDB; облака названы расплывчато (Azure + другие). Оценка по критериям ≈5 из 10</t>
+          <t>«Mature FinOps organization» в вакансии (в посте Kevin — «growing and maturing»); в требованиях Cloudability/CloudHealth — вероятен конкурент; CSDM = ServiceNow CMDB; облака названы расплывчато (Azure + другие). Оценка ≈5 из 10. Письмо Kevin — как к практику: вопрос про актуальность атрибуции владельцев, cross-check рядом с текущим инструментом.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep Rob Fewkes: add WTW to second tier
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -1617,7 +1617,7 @@
           <t>1) Leroy Straker — Director, Cloud Business Office, MetLife (с 02.2026, преемник Rob Fewkes; 11,5 лет в MetLife; в About: Cloud FinOps, TBM, FP&amp;A, FinOps Certified Practitioner; проверено по профилю). Руководитель вакансии и владелец функции.
 2) Patricia Johnson-Clifton — Principal, Cloud Business Office (текущая по LinkedIn-выдаче; на фото рамка Open to work — проверить)
 3) Heather R. (Ratkowiak) — Portfolio Manager, Cloud Business Office (текущая; низкий приоритет)
-Rob Fewkes — НЕ подходит для MetLife: ушёл в WTW 02.2026.</t>
+Rob Fewkes — для MetLife не подходит (ушёл в WTW 02.2026); ведём отдельно как цель в WTW, см. лист «Второй эшелон».</t>
         </is>
       </c>
       <c r="T13" s="43" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="U13" s="43" t="inlineStr">
         <is>
-          <t>Порядок: Leroy, через 3–5 дней Patricia (проверить Open to work). Вопрос в письме — как сейчас делают привязку затрат к приложению/владельцу. Возможный инструмент TBM/FinOps не назван — узнать на звонке (конкурент = второй эшелон). Rob Fewkes в WTW — решить отдельно (консалтинг/брокер исключён по документу).</t>
+          <t>Порядок: Leroy, через 3–5 дней Patricia (проверить Open to work). Вопрос в письме — как сейчас делают привязку затрат к приложению/владельцу. Возможный инструмент TBM/FinOps не назван — узнать на звонке (конкурент = второй эшелон). Rob Fewkes в WTW — решено работать отдельно (лист «Второй эшелон»); в письме ему не упоминать MetLife.</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43359375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="25" min="1" max="1"/>
@@ -4357,8 +4357,35 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1" s="26">
-      <c r="A9" s="52" t="inlineStr">
+    <row r="9" ht="120" customHeight="1" s="26">
+      <c r="A9" s="53" t="inlineStr">
+        <is>
+          <t>WTW</t>
+        </is>
+      </c>
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t>— (вакансии нет, сигнал — должность)</t>
+        </is>
+      </c>
+      <c r="C9" s="55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" s="55" t="inlineStr">
+        <is>
+          <t>Rob Fewkes — Head of Cost Optimization – Global Technology (с 02.2026, 9 мес.; проверено по профилю). До этого 3 года Head of Cloud Business Office в MetLife (прогнозы, облачные расходы). Роль целиком про технологические затраты.</t>
+        </is>
+      </c>
+      <c r="E9" s="55" t="inlineStr">
+        <is>
+          <t>Холодный заход без вакансии; WTW — advisory/брокер (консалтинг по документу исключён, но решено работать с Rob как с внутренним покупателем); облака и бюджет не проверены. В письме не упоминать MetLife и Leroy Straker. Ссылка: https://www.linkedin.com/in/robfewkes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1" s="26">
+      <c r="A10" s="52" t="inlineStr">
         <is>
           <t>Исключены сразу: консалтинг и интеграторы (Deloitte, Accenture, Cognizant, Alvarez &amp; Marsal, TCS, WWT, AHEAD, Synechron), господрядчики (SAIC, Peraton, Booz Allen, MetroStar), кадровые агентства, AI-лаборатории, ServiceNow (конкурент).</t>
         </is>
@@ -5346,7 +5373,7 @@
     <row r="1000" ht="15.75" customHeight="1" s="26"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A10:E10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" display="FinOps Lead - Cloud" r:id="rId1"/>

</xml_diff>

<commit_message>
Add WTW row (Rob Fewkes) to main sheet from user's working copy
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -704,7 +704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:U18"/>
+  <dimension ref="A1:U19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43359375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="25" min="1" max="1"/>
@@ -1617,7 +1617,7 @@
           <t>1) Leroy Straker — Director, Cloud Business Office, MetLife (с 02.2026, преемник Rob Fewkes; 11,5 лет в MetLife; в About: Cloud FinOps, TBM, FP&amp;A, FinOps Certified Practitioner; проверено по профилю). Руководитель вакансии и владелец функции.
 2) Patricia Johnson-Clifton — Principal, Cloud Business Office (текущая по LinkedIn-выдаче; на фото рамка Open to work — проверить)
 3) Heather R. (Ratkowiak) — Portfolio Manager, Cloud Business Office (текущая; низкий приоритет)
-Rob Fewkes — для MetLife не подходит (ушёл в WTW 02.2026); ведём отдельно как цель в WTW, см. лист «Второй эшелон».</t>
+Rob Fewkes — для MetLife не подходит (ушёл в WTW 02.2026); ведём отдельно как цель в WTW, см. строку WTW (№11) в этом листе.</t>
         </is>
       </c>
       <c r="T13" s="43" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="U13" s="43" t="inlineStr">
         <is>
-          <t>Порядок: Leroy, через 3–5 дней Patricia (проверить Open to work). Вопрос в письме — как сейчас делают привязку затрат к приложению/владельцу. Возможный инструмент TBM/FinOps не назван — узнать на звонке (конкурент = второй эшелон). Rob Fewkes в WTW — решено работать отдельно (лист «Второй эшелон»); в письме ему не упоминать MetLife.</t>
+          <t>Порядок: Leroy, через 3–5 дней Patricia (проверить Open to work). Вопрос в письме — как сейчас делают привязку затрат к приложению/владельцу. Возможный инструмент TBM/FinOps не назван — узнать на звонке (конкурент = второй эшелон). Rob Fewkes в WTW — решено работать отдельно (строка WTW №11 в этом листе); в письме ему не упоминать MetLife.</t>
         </is>
       </c>
     </row>
@@ -1920,30 +1920,125 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="26">
-      <c r="B18" s="46" t="inlineStr">
+    <row r="17" ht="120" customHeight="1" s="26">
+      <c r="A17" s="37" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>WTW (Willis Towers Watson)</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="inlineStr">
+        <is>
+          <t>Страховой брокер и консалтинг</t>
+        </is>
+      </c>
+      <c r="D17" s="40" t="inlineStr">
+        <is>
+          <t>AI Economics &amp; FinOps Lead</t>
+        </is>
+      </c>
+      <c r="E17" s="39" t="inlineStr">
+        <is>
+          <t>25.09.2026 (Великобритания)</t>
+        </is>
+      </c>
+      <c r="F17" s="45" t="inlineStr">
+        <is>
+          <t>AWS, Azure, GCP (из вакансии Cloud Security Engineer); основное облако — Azure</t>
+        </is>
+      </c>
+      <c r="G17" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="H17" s="45" t="inlineStr">
+        <is>
+          <t>Модель FinOps уже есть, её развивают; строят FinOps для ИИ и нанимают сразу нескольких человек</t>
+        </is>
+      </c>
+      <c r="I17" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="39" t="inlineStr">
+        <is>
+          <t>Теги, showback/chargeback, владельцы затрат</t>
+        </is>
+      </c>
+      <c r="K17" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="L17" s="45" t="inlineStr">
+        <is>
+          <t>Затраты привязывают к продуктам, платформам и командам-владельцам</t>
+        </is>
+      </c>
+      <c r="M17" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="N17" s="39" t="inlineStr">
+        <is>
+          <t>Reservations, savings plans, использование обязательств</t>
+        </is>
+      </c>
+      <c r="O17" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" s="39" t="inlineStr">
+        <is>
+          <t>Azure Cost Management, Power BI</t>
+        </is>
+      </c>
+      <c r="Q17" s="42">
+        <f>G17+I17+K17+M17+O17</f>
+        <v/>
+      </c>
+      <c r="R17" s="39" t="inlineStr">
+        <is>
+          <t>Не указано. Нанимающий руководитель в США — Rob Fewkes</t>
+        </is>
+      </c>
+      <c r="S17" s="15" t="inlineStr">
+        <is>
+          <t>Rob Fewkes, Head of Cost Optimization</t>
+        </is>
+      </c>
+      <c r="T17" s="15" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/robfewkes/</t>
+        </is>
+      </c>
+      <c r="U17" s="15" t="inlineStr">
+        <is>
+          <t>Сам публикует вакансии своей команды: AI &amp; Cloud FinOps Engineer (11.09, США) и Vendor Performance Management Lead (18.09, США: анализ инструментов, лицензий и лишних расходов). Заходить через расходы на облака и ИИ и их распределение по владельцам. Контакт 3-го круга — писать через InMail или запрос на знакомство. Добавлена 06.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="26"/>
+    <row r="19" ht="15" customHeight="1" s="26">
+      <c r="B19" s="46" t="inlineStr">
         <is>
           <t>Сколько компаний набрали балл по критерию</t>
         </is>
       </c>
-      <c r="G18" s="47">
-        <f>COUNTIF(G7:G16,"&gt;0")</f>
+      <c r="G19" s="47">
+        <f>COUNTIF(G7:G17,"&gt;0")</f>
         <v/>
       </c>
-      <c r="I18" s="47">
-        <f>COUNTIF(I7:I16,"&gt;0")</f>
+      <c r="I19" s="47">
+        <f>COUNTIF(I7:I17,"&gt;0")</f>
         <v/>
       </c>
-      <c r="K18" s="47">
-        <f>COUNTIF(K7:K16,"&gt;0")</f>
+      <c r="K19" s="47">
+        <f>COUNTIF(K7:K17,"&gt;0")</f>
         <v/>
       </c>
-      <c r="M18" s="47">
-        <f>COUNTIF(M7:M16,"&gt;0")</f>
+      <c r="M19" s="47">
+        <f>COUNTIF(M7:M17,"&gt;0")</f>
         <v/>
       </c>
-      <c r="O18" s="47">
-        <f>COUNTIF(O7:O16,"&gt;0")</f>
+      <c r="O19" s="47">
+        <f>COUNTIF(O7:O17,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -4358,31 +4453,11 @@
       </c>
     </row>
     <row r="9" ht="120" customHeight="1" s="26">
-      <c r="A9" s="53" t="inlineStr">
-        <is>
-          <t>WTW</t>
-        </is>
-      </c>
-      <c r="B9" s="54" t="inlineStr">
-        <is>
-          <t>— (вакансии нет, сигнал — должность)</t>
-        </is>
-      </c>
-      <c r="C9" s="55" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D9" s="55" t="inlineStr">
-        <is>
-          <t>Rob Fewkes — Head of Cost Optimization – Global Technology (с 02.2026, 9 мес.; проверено по профилю). До этого 3 года Head of Cloud Business Office в MetLife (прогнозы, облачные расходы). Роль целиком про технологические затраты.</t>
-        </is>
-      </c>
-      <c r="E9" s="55" t="inlineStr">
-        <is>
-          <t>Холодный заход без вакансии; WTW — advisory/брокер (консалтинг по документу исключён, но решено работать с Rob как с внутренним покупателем); облака и бюджет не проверены. В письме не упоминать MetLife и Leroy Straker. Ссылка: https://www.linkedin.com/in/robfewkes</t>
-        </is>
-      </c>
+      <c r="A9" s="53" t="n"/>
+      <c r="B9" s="54" t="n"/>
+      <c r="C9" s="55" t="n"/>
+      <c r="D9" s="55" t="n"/>
+      <c r="E9" s="55" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1" s="26">
       <c r="A10" s="52" t="inlineStr">

</xml_diff>

<commit_message>
Add Edward Jones candidate contacts from Seamless
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR5sk9Sdjz8zJLFvXqXRxv
</commit_message>
<xml_diff>
--- a/FinOps_contacts_LinkedIn.xlsx
+++ b/FinOps_contacts_LinkedIn.xlsx
@@ -4424,7 +4424,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="150" customHeight="1" s="26">
+    <row r="8" ht="260" customHeight="1" s="26">
       <c r="A8" s="53" t="inlineStr">
         <is>
           <t>Edward Jones</t>
@@ -4443,7 +4443,14 @@
       <c r="D8" s="55" t="inlineStr">
         <is>
           <t>Fortune 500, 20 000 консультантов, St. Louis; крупные облачные расходы; роль: распределение затрат, showback/chargeback, коммитменты (reservations, savings plans), service owners и CSDM.
-Контакт: Kevin Krueger — Head of Cloud Business Office (с 08.2024; 10+ лет FinOps/TBM; сам нанимает на «growing and maturing FinOps program»; проверено по профилю). Репостнул вакансию Managing Director, Head of Cloud — возможно, его руководитель.</t>
+Контакт: Kevin Krueger — Head of Cloud Business Office (с 08.2024; 10+ лет FinOps/TBM; сам нанимает на «growing and maturing FinOps program»; проверено по профилю). Репостнул вакансию Managing Director, Head of Cloud — возможно, его руководитель.
+Ссылка Kevin Krueger: https://www.linkedin.com/in/kevinbkrueger
+Кандидаты из Seamless (не проверены по профилям):
+• Rushil Chugh — Head of Cloud Operations: https://www.linkedin.com/in/crushil
+• Mashud Qayum — Finance Team Leader, Technology: https://www.linkedin.com/in/mashud-qayum-b3108447
+• Sareema Koirala Phillips — Senior Financial Analyst (IT Finance): https://www.linkedin.com/in/sareema-koirala-phillips-6971152a
+• Aaron Dixon — Digital Product Owner, Cloud Platform Engineering: https://www.linkedin.com/in/aaron-dixon
+Не найдены: Managing Director, Head of Cloud; Technology Business Manager.</t>
         </is>
       </c>
       <c r="E8" s="55" t="inlineStr">

</xml_diff>